<commit_message>
adding compliance metadata to third-party assets
</commit_message>
<xml_diff>
--- a/Production/AssetRegistry/AssetRegistry.xlsx
+++ b/Production/AssetRegistry/AssetRegistry.xlsx
@@ -13,14 +13,14 @@
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="116">
   <si>
     <t xml:space="preserve">BLACKOUT ASSET REGISTRY</t>
   </si>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">https://fab.com/s/cf1650818637</t>
   </si>
   <si>
-    <t xml:space="preserve">Fab Standard License (Licenses/Fab.pdf)</t>
+    <t xml:space="preserve">Creative Commons Attribution (CC BY 4.0 – Production/Licenses/CC4.txt)</t>
   </si>
   <si>
     <t xml:space="preserve">Free</t>
@@ -95,6 +95,9 @@
   </si>
   <si>
     <t xml:space="preserve">5.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production/Evidences/TP-0001</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -148,7 +151,7 @@
     <t xml:space="preserve">https://fab.com/s/cc3b4087041e</t>
   </si>
   <si>
-    <t xml:space="preserve">Creative Common Attribution (CC BY 4.0 – Licenses/CC4.pdf)</t>
+    <t xml:space="preserve">Production/Evidences/TP-0002</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
@@ -172,7 +175,13 @@
     <t xml:space="preserve">https://fab.com/s/7b469fce462f</t>
   </si>
   <si>
-    <t xml:space="preserve">Date of acquisition is estimated based on addition commit (fa43e8b1); Arch and Wall meshes had their origin adjusted; Wall mesh was resized</t>
+    <t xml:space="preserve">Fab Standard License (Production/Licenses/Fab.pdf)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production/Evidences/TP-0003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date of acquisition is estimated based on addition commit (fa43e8b1); Arch and Wall meshes had their origin adjusted; Wall mesh was resized. Although acquired without any costs on the recorded date, this asset is now accessible only through a purchase</t>
   </si>
   <si>
     <t xml:space="preserve">TP-0004</t>
@@ -187,6 +196,9 @@
     <t xml:space="preserve">https://fab.com/s/75397d4851d0</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0004</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date of acquisition is estimated based on addition commit (9ec4bb36); Handle stands removed</t>
   </si>
   <si>
@@ -202,6 +214,9 @@
     <t xml:space="preserve">https://fab.com/s/2ef2c717b36a</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0005</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date of acquisition is estimated based on addition commit (9ec4bb36); All objects removed from original fbx but the one actually used in the project</t>
   </si>
   <si>
@@ -214,35 +229,13 @@
     <t xml:space="preserve">Quixel Megascans</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">https://fab.com/s/c68116d204a8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">https://fab.com/s/c7859152ef31</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Date of acquisition is estimated based on addition commit (da70e717); For some reason there are two urls where this asset can be found. Aside for technical details, it’s not really possible to determine which one is being used in the project as of today. Therefore, both links are being provided</t>
+    <t xml:space="preserve">https://fab.com/s/c68116d204a8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production/Evidences/TP-0006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date of acquisition is estimated based on addition commit (da70e717)</t>
   </si>
   <si>
     <t xml:space="preserve">TP-0007</t>
@@ -257,13 +250,13 @@
     <t xml:space="preserve">https://fab.com/s/59bcbbec347a</t>
   </si>
   <si>
-    <t xml:space="preserve">Date of acquisition is estimated based on addition commit (da70e717)</t>
+    <t xml:space="preserve">Production/Evidences/TP-0007</t>
   </si>
   <si>
     <t xml:space="preserve">TP-0008</t>
   </si>
   <si>
-    <t xml:space="preserve">Fire effect</t>
+    <t xml:space="preserve">Starter content</t>
   </si>
   <si>
     <t xml:space="preserve">Material/sound wave</t>
@@ -278,7 +271,7 @@
     <t xml:space="preserve">Engine content</t>
   </si>
   <si>
-    <t xml:space="preserve">Unreal Engine EULA (Licenses/UnrealEngineEULA.pdf)</t>
+    <t xml:space="preserve">Unreal Engine EULA (Production/Licenses/UnrealEngineEULA.pdf)</t>
   </si>
   <si>
     <t xml:space="preserve">Added to project through engine’s “Add feature or content pack” option</t>
@@ -287,6 +280,9 @@
     <t xml:space="preserve">5.6</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0008</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date of acquisition is estimated based on addition commit (47ca336a)</t>
   </si>
   <si>
@@ -314,6 +310,9 @@
     <t xml:space="preserve">N/A</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0009</t>
+  </si>
+  <si>
     <t xml:space="preserve">Origin of previous sfx not found. Using this effect instead</t>
   </si>
   <si>
@@ -329,7 +328,10 @@
     <t xml:space="preserve">https://freesound.org/s/770346/</t>
   </si>
   <si>
-    <t xml:space="preserve">Creative Common 0 (Licences/CC0.pdf)</t>
+    <t xml:space="preserve">Creative Commons 0 (Production/Licenses/CC0.pdf)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production/Evidences/TP-0010</t>
   </si>
   <si>
     <t xml:space="preserve">TP-0011</t>
@@ -344,6 +346,9 @@
     <t xml:space="preserve">https://freesound.org/s/274200/</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0011</t>
+  </si>
+  <si>
     <t xml:space="preserve">TP-0012</t>
   </si>
   <si>
@@ -356,6 +361,9 @@
     <t xml:space="preserve">https://fab.com/s/5564160d337f</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0012</t>
+  </si>
+  <si>
     <t xml:space="preserve">TP-0013</t>
   </si>
   <si>
@@ -368,6 +376,9 @@
     <t xml:space="preserve">https://fab.com/s/c039e3862941</t>
   </si>
   <si>
+    <t xml:space="preserve">Production/Evidences/TP-0013</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date of acquisition is estimated based on addition commit (eec93dcd)</t>
   </si>
   <si>
@@ -384,6 +395,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://fab.com/s/1bc4ef4e6dab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production/Evidences/TP-0014</t>
   </si>
   <si>
     <t xml:space="preserve">Date of acquisition is estimated based on addition commit (c3df3c7b)</t>
@@ -397,7 +411,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -445,12 +459,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -494,7 +502,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -516,10 +524,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -777,34 +781,37 @@
       <c r="K4" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L4" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="M4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>22</v>
@@ -818,34 +825,37 @@
       <c r="K5" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L5" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="M5" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="65.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>22</v>
@@ -859,34 +869,37 @@
       <c r="K6" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L6" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="M6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>22</v>
@@ -900,34 +913,37 @@
       <c r="K7" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L7" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="M7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>22</v>
@@ -941,34 +957,37 @@
       <c r="K8" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L8" s="1" t="s">
+        <v>53</v>
+      </c>
       <c r="M8" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="54.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>53</v>
+      <c r="F9" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>22</v>
@@ -982,34 +1001,37 @@
       <c r="K9" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L9" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="M9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>22</v>
@@ -1023,34 +1045,37 @@
       <c r="K10" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L10" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="M10" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>22</v>
@@ -1059,39 +1084,42 @@
         <v>46225</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>22</v>
@@ -1100,39 +1128,42 @@
         <v>46239</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="D13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="F13" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>22</v>
@@ -1141,36 +1172,39 @@
         <v>46239</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>22</v>
@@ -1179,36 +1213,39 @@
         <v>46237</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>22</v>
@@ -1222,34 +1259,37 @@
       <c r="K15" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L15" s="1" t="s">
+        <v>102</v>
+      </c>
       <c r="M15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>22</v>
@@ -1263,34 +1303,37 @@
       <c r="K16" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L16" s="1" t="s">
+        <v>107</v>
+      </c>
       <c r="M16" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="32.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>22</v>
@@ -1304,11 +1347,14 @@
       <c r="K17" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="L17" s="1" t="s">
+        <v>114</v>
+      </c>
       <c r="M17" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1316,11 +1362,11 @@
     <mergeCell ref="A1:N2"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPágina &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>